<commit_message>
upload essential Rmd docs
</commit_message>
<xml_diff>
--- a/tables/MGWR_var.xlsx
+++ b/tables/MGWR_var.xlsx
@@ -44,7 +44,7 @@
     <t>illum vol density</t>
   </si>
   <si>
-    <t>Illuminated Building Volume Density: Illuminated building footprint volume per hm² within ward, masked by residential area</t>
+    <t>Illuminated Building Volume Density: Illuminated building footprint volume per hectare within ward, masked by residential area</t>
   </si>
   <si>
     <t>Available from band=['built characteristics Class Table']</t>
@@ -66,22 +66,22 @@
     <t>VIIRS Nighttime Day/Night Annual Band Composites V2.2 (2022-2024)</t>
   </si>
   <si>
-    <t>poi kde</t>
-  </si>
-  <si>
-    <t>POI Kernel Density：Mean POI kernel density within ward, masked by residential area</t>
+    <t>POI KD</t>
+  </si>
+  <si>
+    <t>POI Kernel Density: Mean POI kernel density within ward, masked by residential area</t>
   </si>
   <si>
     <t>Available from OSM POI (amenity=*)</t>
   </si>
   <si>
-    <t>OpenSteetMap (2025)</t>
+    <t>OpenStreetMap (2025)</t>
   </si>
   <si>
     <t>POP density</t>
   </si>
   <si>
-    <t>Pop Density: Population density per hm² within ward</t>
+    <t>Pop Density: Population density per hectare within ward</t>
   </si>
   <si>
     <t>Available from col=['POP']</t>

</xml_diff>